<commit_message>
Dyes data part1 added
</commit_message>
<xml_diff>
--- a/master_data_template.xlsx
+++ b/master_data_template.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Downloads\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BD012F9-FE6E-4DB3-B307-7C6B1591EA2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4EB9774-F555-4389-A98A-0DC507DD8D1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Papers Master List" sheetId="1" r:id="rId1"/>
     <sheet name="Metal_Data_raw" sheetId="2" r:id="rId2"/>
-    <sheet name="Data Dictionary" sheetId="3" r:id="rId3"/>
+    <sheet name="Dye_Data_Raw" sheetId="4" r:id="rId3"/>
+    <sheet name="Data Dictionary" sheetId="3" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="776" uniqueCount="284">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1327" uniqueCount="463">
   <si>
     <t>paper_id</t>
   </si>
@@ -888,13 +889,550 @@
   </si>
   <si>
     <t>qe_exp from kinetics Table 2; MAB (activated biochar)[cite: 18]</t>
+  </si>
+  <si>
+    <t>Dyes Papers</t>
+  </si>
+  <si>
+    <t>P020</t>
+  </si>
+  <si>
+    <t>Comparative adsorption isotherms and modeling of methylene blue onto activated carbons</t>
+  </si>
+  <si>
+    <t>Belhachemi, Addoun</t>
+  </si>
+  <si>
+    <t>Applied Water Science</t>
+  </si>
+  <si>
+    <t>10.1007/s13201-011-0014-1</t>
+  </si>
+  <si>
+    <t>MB</t>
+  </si>
+  <si>
+    <t>P020_Belhachemi2011.pdf</t>
+  </si>
+  <si>
+    <t>P021</t>
+  </si>
+  <si>
+    <t>Experimental Design, Equilibrium Modeling and Kinetic Studies on the Adsorption of Methylene Blue by Adsorbent: Activated Carbon from Durian Shell Waste</t>
+  </si>
+  <si>
+    <t>Tran, Ðo, Ha, Duong, Chu, Vu, Chau, Tran, Song</t>
+  </si>
+  <si>
+    <t>10.3390/ma15238566</t>
+  </si>
+  <si>
+    <t>P021_Tran2022.pdf</t>
+  </si>
+  <si>
+    <t>P022</t>
+  </si>
+  <si>
+    <t>Assessment of the Porous Structure and Surface Chemistry of Activated Biocarbons Used for Methylene Blue Adsorption</t>
+  </si>
+  <si>
+    <t>Charmas, Ziezio, Jedynak</t>
+  </si>
+  <si>
+    <t>10.3390/molecules28134922</t>
+  </si>
+  <si>
+    <t>P022_Charmas2023.pdf</t>
+  </si>
+  <si>
+    <t>P023</t>
+  </si>
+  <si>
+    <t>Adsorption of methylene blue onto activated carbon produced from tea (Camellia sinensis L.) seed shells: kinetics, equilibrium, and thermodynamics studies</t>
+  </si>
+  <si>
+    <t>(PMC3709070)</t>
+  </si>
+  <si>
+    <t>Full text not accessible — PMC blocked by CAPTCHA. Abstract gives BET=1530.67 m²/g, pore volume=0.7826 cm³/g, Langmuir qmax=324.7 mg/g, but no C0/pH/dose/time condition-set data confirmable.</t>
+  </si>
+  <si>
+    <t>P023_TeaSeedShell.pdf</t>
+  </si>
+  <si>
+    <t>P024</t>
+  </si>
+  <si>
+    <t>Methylene blue adsorption mechanism of activated carbon synthesised from cashew nut shells</t>
+  </si>
+  <si>
+    <t>(PMC9037662)</t>
+  </si>
+  <si>
+    <t>Full text not accessible — PMC blocked by CAPTCHA.</t>
+  </si>
+  <si>
+    <t>P024_CashewNutShell.pdf</t>
+  </si>
+  <si>
+    <t>P025</t>
+  </si>
+  <si>
+    <t>The Use of High Surface Area Mesoporous-Activated Carbon from Longan Seed Biomass for Increasing Capacity and Kinetics of Methylene Blue Adsorption</t>
+  </si>
+  <si>
+    <t>(PMC8587158)</t>
+  </si>
+  <si>
+    <t>Full text not accessible — PMC blocked by CAPTCHA. Abstract gives BET=1773 m²/g, mesopore volume=0.474 cm³/g, qmax up to 1000 mg/g, but no condition-set data confirmable.</t>
+  </si>
+  <si>
+    <t>P025_LonganSeed.pdf</t>
+  </si>
+  <si>
+    <t>P026</t>
+  </si>
+  <si>
+    <t>Synthesis and characterization of modified activated carbon (MgO/AC) for methylene blue adsorption</t>
+  </si>
+  <si>
+    <t>Not confirmed (not fetched)</t>
+  </si>
+  <si>
+    <t>Water Science &amp; Technology (IWA)</t>
+  </si>
+  <si>
+    <t>Primary adsorbent is a metal-oxide composite (MgO/AC), out of project scope (AC only), consistent with the same exclusion rule applied to metal-oxide composites in the Cd(II) batch. Not fetched further.</t>
+  </si>
+  <si>
+    <t>P026_MgOAC.pdf</t>
+  </si>
+  <si>
+    <t>date stones</t>
+  </si>
+  <si>
+    <t>Langmuir Q0 from Table 3; C0 unstated (isotherm series 30-1000 mg/L)</t>
+  </si>
+  <si>
+    <t>durian shell</t>
+  </si>
+  <si>
+    <t>Langmuir qmax; Dose calculated from 0.05g/20mL</t>
+  </si>
+  <si>
+    <t>qe_exp from pseudo-second order kinetics table (Table 7)</t>
+  </si>
+  <si>
+    <t>wheat bran</t>
+  </si>
+  <si>
+    <t>AC-1; Langmuir qm_calc from Table 7; Elemental from EDX (wt%)</t>
+  </si>
+  <si>
+    <t>AC-1_MW; Langmuir qm_calc from Table 7</t>
+  </si>
+  <si>
+    <t>AC-1-OX; Langmuir qm_calc from Table 7</t>
+  </si>
+  <si>
+    <t>AC-1-OX_MW; Langmuir qm_calc from Table 7</t>
+  </si>
+  <si>
+    <t>AC-2; Langmuir qm_calc from Table 7</t>
+  </si>
+  <si>
+    <t>AC-2_MW; Langmuir qm_calc from Table 7</t>
+  </si>
+  <si>
+    <t>tea seed shells</t>
+  </si>
+  <si>
+    <t>qe_exp from kinetics Table 3; Time approximated from text</t>
+  </si>
+  <si>
+    <t>Langmuir qmax from Table 4</t>
+  </si>
+  <si>
+    <t>cashew nut shells</t>
+  </si>
+  <si>
+    <t>Approximate qe read from Fig 4B at 100 min; properties for AC activated at 850 C</t>
+  </si>
+  <si>
+    <t>longan seed</t>
+  </si>
+  <si>
+    <t>Sample A1; Langmuir qm from Table 7</t>
+  </si>
+  <si>
+    <t>Sample A2; Langmuir qm from Table 7</t>
+  </si>
+  <si>
+    <t>Sample A3; Langmuir qm from Table 7</t>
+  </si>
+  <si>
+    <t>Sample A4; Langmuir qm from Table 7</t>
+  </si>
+  <si>
+    <t>Sample A5; Langmuir qm from Table 7</t>
+  </si>
+  <si>
+    <t>Sample A6; Langmuir qm from Table 7</t>
+  </si>
+  <si>
+    <t>walnut shell</t>
+  </si>
+  <si>
+    <t>Extracted only plain AC per instructions; Optimal conditions from Table 4; Internal inconsistency noted between stated % removal and tabulated qe</t>
+  </si>
+  <si>
+    <t>P027</t>
+  </si>
+  <si>
+    <t>Kinetic and Thermodynamic Study of Methylene Blue Adsorption onto Activated Carbon Obtained from the Peel of musa paradisiaca</t>
+  </si>
+  <si>
+    <t>Vallejo, Diaz-Uribe, Duran, Vargas-Delgadillo, Barbosa</t>
+  </si>
+  <si>
+    <t>Sci (MDPI)</t>
+  </si>
+  <si>
+    <t>10.3390/sci7040170</t>
+  </si>
+  <si>
+    <t>P027_Vallejo2025.pdf</t>
+  </si>
+  <si>
+    <t>P028</t>
+  </si>
+  <si>
+    <t>Adsorption of methylene blue onto activated carbon produced from tea (Camellia sinensis L.) seed shells</t>
+  </si>
+  <si>
+    <t>Full text not accessible — PMC blocked by CAPTCHA (repeat candidate from Batch 1).</t>
+  </si>
+  <si>
+    <t>P028_TeaSeedShell.pdf</t>
+  </si>
+  <si>
+    <t>P029</t>
+  </si>
+  <si>
+    <t>Adsorption of phenol and methylene blue contaminants onto high-performance catalytic activated carbon from biomass residues</t>
+  </si>
+  <si>
+    <t>2025 (collection date)</t>
+  </si>
+  <si>
+    <t>(PMC11721239)</t>
+  </si>
+  <si>
+    <t>MB (binary system with phenol)</t>
+  </si>
+  <si>
+    <t>Full text not accessible — PMC blocked by CAPTCHA. Abstract gives only combined single/binary qmax ranges (352.25–855.96 mg/g single; 348.90–456.39 mg/g binary), no BET/pore volume or condition-set data confirmable.</t>
+  </si>
+  <si>
+    <t>P029_PhenolMBCatalyticAC.pdf</t>
+  </si>
+  <si>
+    <t>P030</t>
+  </si>
+  <si>
+    <t>Experiments and physical investigation on the adsorption of methylene [blue] on activated carbon</t>
+  </si>
+  <si>
+    <t>(PMC12749830)</t>
+  </si>
+  <si>
+    <t>P030_PhysicalInvestigationAC.pdf</t>
+  </si>
+  <si>
+    <t>P031</t>
+  </si>
+  <si>
+    <t>Adsorption of Methylene Blue on Activated Carbon Surfaces Obtained by Shock Compression of Graphite Using Reactive Molecular Dynamics</t>
+  </si>
+  <si>
+    <t>(PMC11679267, MDPI)</t>
+  </si>
+  <si>
+    <t>This is a molecular dynamics simulation study, not an empirical batch-adsorption experiment — no real C0/pH/dose/time/BET data to extract regardless of access. Out of scope for a literature-derived experimental dataset.</t>
+  </si>
+  <si>
+    <t>P031_MDSimulationGraphiteAC.pdf</t>
+  </si>
+  <si>
+    <t>P032</t>
+  </si>
+  <si>
+    <t>Kinetics and Thermodynamics Study of Methylene Blue Adsorption to Sucrose- and Urea-Derived Nitrogen-Enriched, Hierarchically Porous Carbon Activated by KOH and H3PO4</t>
+  </si>
+  <si>
+    <t>Not confirmed (ACS blocked)</t>
+  </si>
+  <si>
+    <t>10.1021/acsomega.3c00339</t>
+  </si>
+  <si>
+    <t>Full text not accessible — ACS Publications blocks automated fetch (bot detection); PMC mirror (PMC10173434) blocked by CAPTCHA.</t>
+  </si>
+  <si>
+    <t>P032_SucroseUreaNC.pdf</t>
+  </si>
+  <si>
+    <t>P033</t>
+  </si>
+  <si>
+    <t>Kinetic and Thermodynamic Studies of Methylene Blue Adsorption on Biomass-Derived Biocarbon Materials</t>
+  </si>
+  <si>
+    <t>(PMC12985126)</t>
+  </si>
+  <si>
+    <t>Full text not accessible — PMC blocked by CAPTCHA. Abstract gives BET range (109–154 m²/g) but no condition-set data confirmable.</t>
+  </si>
+  <si>
+    <t>P033_BiomassBiocarbon.pdf</t>
+  </si>
+  <si>
+    <t>banana peel</t>
+  </si>
+  <si>
+    <t>qe_exp from pseudo-second order kinetics (Table 3)[cite: 33]</t>
+  </si>
+  <si>
+    <t>AC/EDTA; qe_exp from pseudo-second order kinetics (Table 3)[cite: 33]</t>
+  </si>
+  <si>
+    <t>AC/TA; qe_exp from pseudo-second order kinetics (Table 3)[cite: 33]</t>
+  </si>
+  <si>
+    <t>AC/CA; qe_exp from pseudo-second order kinetics (Table 3)[cite: 33]</t>
+  </si>
+  <si>
+    <t>Langmuir qmax from Table 4[cite: 33]</t>
+  </si>
+  <si>
+    <t>AC/EDTA; Langmuir qmax from Table 4.Cont[cite: 33]</t>
+  </si>
+  <si>
+    <t>AC/TA; Langmuir qmax from Table 4.Cont[cite: 33]</t>
+  </si>
+  <si>
+    <t>AC/CA; Langmuir qmax from Table 4.Cont[cite: 33]</t>
+  </si>
+  <si>
+    <t>Langmuir qmax from Table 4 (Duplicate of paper P023)</t>
+  </si>
+  <si>
+    <t>qe_exp from kinetics Table 3 (Duplicate of paper P023)</t>
+  </si>
+  <si>
+    <t>Moringa oleifera husk</t>
+  </si>
+  <si>
+    <t>Langmuir qm (Table 4) for MBMHC</t>
+  </si>
+  <si>
+    <t>sesame husk</t>
+  </si>
+  <si>
+    <t>Langmuir qm (Table 4) for MBSHC</t>
+  </si>
+  <si>
+    <t>baobab husk</t>
+  </si>
+  <si>
+    <t>Langmuir qm (Table 4) for MBBHC</t>
+  </si>
+  <si>
+    <t>Fitted PSO qe (Table 3) for MBMHC single-solute system</t>
+  </si>
+  <si>
+    <t>Fitted PSO qe (Table 3) for MBSHC single-solute system</t>
+  </si>
+  <si>
+    <t>Fitted PSO qe (Table 3) for MBBHC single-solute system</t>
+  </si>
+  <si>
+    <t>olive waste</t>
+  </si>
+  <si>
+    <t>Langmuir qmax (Table 2) - Note: Massive internal inconsistency; graph shows capacities up to ~240 mg/g. Value recorded exactly as tabulated.</t>
+  </si>
+  <si>
+    <t>Modeled Qm from Multilayer Model (Table 4)</t>
+  </si>
+  <si>
+    <t>qe_exp from kinetics (Table 3); Dose calculated from 0.2g in 50mL</t>
+  </si>
+  <si>
+    <t>sucrose and urea polymer</t>
+  </si>
+  <si>
+    <t>SU-KOH; qe_exp from kinetics Table 1; XPS atomic % only, no bulk wt% reported</t>
+  </si>
+  <si>
+    <t>text</t>
+  </si>
+  <si>
+    <t>SU-KOH; Langmuir Qmax</t>
+  </si>
+  <si>
+    <t>SU-KOH; Table 6 maximum capacity</t>
+  </si>
+  <si>
+    <t>SU-H3PO4; qe_exp from kinetics Table 1; XPS atomic % only, no bulk wt% reported</t>
+  </si>
+  <si>
+    <t>SU-H3PO4; Langmuir Qmax</t>
+  </si>
+  <si>
+    <t>SU-H3PO4; Table 6 maximum capacity</t>
+  </si>
+  <si>
+    <t>P034</t>
+  </si>
+  <si>
+    <t>Efficient adsorptive removal of Congo Red dye using activated carbon derived from Spathodea campanulata flowers</t>
+  </si>
+  <si>
+    <t>Sudarsan, Murugesan, Varadavenkatesan, Vinayagam, Selvaraj</t>
+  </si>
+  <si>
+    <t>Scientific Reports</t>
+  </si>
+  <si>
+    <t>10.1038/s41598-025-86032-9</t>
+  </si>
+  <si>
+    <t>CR</t>
+  </si>
+  <si>
+    <t>P034_Sudarsan2025.pdf</t>
+  </si>
+  <si>
+    <t>P035</t>
+  </si>
+  <si>
+    <t>Twigs-derived activated carbons via H3PO4/ZnCl2 composite activation for methylene blue and congo red dyes removal</t>
+  </si>
+  <si>
+    <t>Zubir, Zaini</t>
+  </si>
+  <si>
+    <t>10.1038/s41598-020-71034-6</t>
+  </si>
+  <si>
+    <t>CR, MB</t>
+  </si>
+  <si>
+    <t>P035_Zubir2020.pdf</t>
+  </si>
+  <si>
+    <t>P036</t>
+  </si>
+  <si>
+    <t>Efficient Removal of Congo Red from Wastewater Using Date-Pit Activated Carbon</t>
+  </si>
+  <si>
+    <t>Fibers and Polymers (Springer)</t>
+  </si>
+  <si>
+    <t>10.1007/s12221-025-01277-5</t>
+  </si>
+  <si>
+    <t>Not yet fetched for full text — Fibers and Polymers is a standard (non-open-access) Springer journal, unlike SpringerOpen/Applied Water Science; likely paywalled. Abstract gives BET=946.68 m²/g, pore volume=0.46 cm³/g but no condition-set data confirmable at this access level.</t>
+  </si>
+  <si>
+    <t>P036_DatePitAC.pdf</t>
+  </si>
+  <si>
+    <t>P037</t>
+  </si>
+  <si>
+    <t>Adsorption characteristics of Congo Red on coal-based mesoporous activated carbon</t>
+  </si>
+  <si>
+    <t>Adsorption Science &amp; Technology (ScienceDirect)</t>
+  </si>
+  <si>
+    <t>ScienceDirect abstract-page only (robots-disallowed for full fetch); reports BET range 331–679 m²/g and pHpzc &gt;10 across several ACs but no accessible condition-set data.</t>
+  </si>
+  <si>
+    <t>P037_CoalMesoporousAC.pdf</t>
+  </si>
+  <si>
+    <t>P038</t>
+  </si>
+  <si>
+    <t>Adsorption of congo red on mesoporous activated carbon prepared by CO2 physical activation</t>
+  </si>
+  <si>
+    <t>Chinese Journal of Chemical Engineering (ScienceDirect)</t>
+  </si>
+  <si>
+    <t>CR (also Amido Black 10B)</t>
+  </si>
+  <si>
+    <t>ScienceDirect blocks full fetch (robots disallowed). Abstract reports max qe=559.3 mg/g for CR but no BET/pore volume/condition-set data at abstract level.</t>
+  </si>
+  <si>
+    <t>P038_SargassumCO2AC.pdf</t>
+  </si>
+  <si>
+    <t>P039</t>
+  </si>
+  <si>
+    <t>Adsorption enhancement of Congo red dye from wastewater based on edamame shell originated activated carbon by the cations</t>
+  </si>
+  <si>
+    <t>Diamond and Related Materials (ScienceDirect)</t>
+  </si>
+  <si>
+    <t>ScienceDirect blocks full fetch. Abstract reports an unusually high qmax (1509.60 mg/g) but no accessible BET/pore-volume/condition-set numbers to verify or extract.</t>
+  </si>
+  <si>
+    <t>P039_EdamameShellAC.pdf</t>
+  </si>
+  <si>
+    <t>fennel seeds</t>
+  </si>
+  <si>
+    <t>FS5; Langmuir qm from Table 3</t>
+  </si>
+  <si>
+    <t>caraway seeds</t>
+  </si>
+  <si>
+    <t>CS5; Langmuir qm from Table 3</t>
+  </si>
+  <si>
+    <t>FS6; Langmuir qm from Table 3</t>
+  </si>
+  <si>
+    <t>CS6; Langmuir qm from Table 3</t>
+  </si>
+  <si>
+    <t>FS5; qe_exp from kinetics Table 5; Ce calculated</t>
+  </si>
+  <si>
+    <t>CS5; qe_exp from kinetics Table 5; Ce calculated</t>
+  </si>
+  <si>
+    <t>FS6; qe_exp from kinetics Table 5; Ce calculated</t>
+  </si>
+  <si>
+    <t>CS6; qe_exp from kinetics Table 5; Ce calculated</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -940,8 +1478,15 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -952,6 +1497,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF2F5496"/>
         <bgColor rgb="FF666699"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -982,7 +1539,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -999,6 +1556,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1263,7 +1823,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M20"/>
+  <dimension ref="A1:M41"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -1314,8 +1874,8 @@
         <v>10</v>
       </c>
       <c r="M1" s="3">
-        <f>COUNTIF(H2:H500,"Y")</f>
-        <v>5</v>
+        <f>COUNTIF(H2:H499,"Y")</f>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
@@ -1353,8 +1913,8 @@
         <v>13</v>
       </c>
       <c r="M2" s="3">
-        <f>COUNTIF(H2:H500,"N")</f>
-        <v>9</v>
+        <f>COUNTIF(H2:H499,"N")</f>
+        <v>23</v>
       </c>
     </row>
     <row r="3" spans="1:13" ht="57.6" x14ac:dyDescent="0.3">
@@ -1931,14 +2491,659 @@
       </c>
       <c r="J20" s="7"/>
     </row>
+    <row r="21" spans="1:10" s="8" customFormat="1" ht="25.8" x14ac:dyDescent="0.5">
+      <c r="B21" s="9" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="22" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>285</v>
+      </c>
+      <c r="B22" t="s">
+        <v>286</v>
+      </c>
+      <c r="C22" t="s">
+        <v>287</v>
+      </c>
+      <c r="D22">
+        <v>2011</v>
+      </c>
+      <c r="E22" t="s">
+        <v>288</v>
+      </c>
+      <c r="F22" t="s">
+        <v>289</v>
+      </c>
+      <c r="G22" t="s">
+        <v>290</v>
+      </c>
+      <c r="H22" t="s">
+        <v>12</v>
+      </c>
+      <c r="I22" t="s">
+        <v>90</v>
+      </c>
+      <c r="J22" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="23" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>292</v>
+      </c>
+      <c r="B23" t="s">
+        <v>293</v>
+      </c>
+      <c r="C23" t="s">
+        <v>294</v>
+      </c>
+      <c r="D23">
+        <v>2022</v>
+      </c>
+      <c r="E23" t="s">
+        <v>101</v>
+      </c>
+      <c r="F23" t="s">
+        <v>295</v>
+      </c>
+      <c r="G23" t="s">
+        <v>290</v>
+      </c>
+      <c r="H23" t="s">
+        <v>12</v>
+      </c>
+      <c r="I23" t="s">
+        <v>90</v>
+      </c>
+      <c r="J23" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>297</v>
+      </c>
+      <c r="B24" t="s">
+        <v>298</v>
+      </c>
+      <c r="C24" t="s">
+        <v>299</v>
+      </c>
+      <c r="D24">
+        <v>2023</v>
+      </c>
+      <c r="E24" t="s">
+        <v>128</v>
+      </c>
+      <c r="F24" t="s">
+        <v>300</v>
+      </c>
+      <c r="G24" t="s">
+        <v>290</v>
+      </c>
+      <c r="H24" t="s">
+        <v>12</v>
+      </c>
+      <c r="I24" t="s">
+        <v>90</v>
+      </c>
+      <c r="J24" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>302</v>
+      </c>
+      <c r="B25" t="s">
+        <v>303</v>
+      </c>
+      <c r="C25" t="s">
+        <v>233</v>
+      </c>
+      <c r="D25" t="s">
+        <v>235</v>
+      </c>
+      <c r="E25" t="s">
+        <v>304</v>
+      </c>
+      <c r="F25" t="s">
+        <v>235</v>
+      </c>
+      <c r="G25" t="s">
+        <v>290</v>
+      </c>
+      <c r="H25" t="s">
+        <v>103</v>
+      </c>
+      <c r="I25" t="s">
+        <v>305</v>
+      </c>
+      <c r="J25" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>307</v>
+      </c>
+      <c r="B26" t="s">
+        <v>308</v>
+      </c>
+      <c r="C26" t="s">
+        <v>233</v>
+      </c>
+      <c r="D26" t="s">
+        <v>235</v>
+      </c>
+      <c r="E26" t="s">
+        <v>309</v>
+      </c>
+      <c r="F26" t="s">
+        <v>235</v>
+      </c>
+      <c r="G26" t="s">
+        <v>290</v>
+      </c>
+      <c r="H26" t="s">
+        <v>103</v>
+      </c>
+      <c r="I26" t="s">
+        <v>310</v>
+      </c>
+      <c r="J26" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>312</v>
+      </c>
+      <c r="B27" t="s">
+        <v>313</v>
+      </c>
+      <c r="C27" t="s">
+        <v>233</v>
+      </c>
+      <c r="D27" t="s">
+        <v>235</v>
+      </c>
+      <c r="E27" t="s">
+        <v>314</v>
+      </c>
+      <c r="F27" t="s">
+        <v>235</v>
+      </c>
+      <c r="G27" t="s">
+        <v>290</v>
+      </c>
+      <c r="H27" t="s">
+        <v>103</v>
+      </c>
+      <c r="I27" t="s">
+        <v>315</v>
+      </c>
+      <c r="J27" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>317</v>
+      </c>
+      <c r="B28" t="s">
+        <v>318</v>
+      </c>
+      <c r="C28" t="s">
+        <v>319</v>
+      </c>
+      <c r="D28" t="s">
+        <v>235</v>
+      </c>
+      <c r="E28" t="s">
+        <v>320</v>
+      </c>
+      <c r="F28" t="s">
+        <v>235</v>
+      </c>
+      <c r="G28" t="s">
+        <v>290</v>
+      </c>
+      <c r="H28" t="s">
+        <v>103</v>
+      </c>
+      <c r="I28" t="s">
+        <v>321</v>
+      </c>
+      <c r="J28" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>349</v>
+      </c>
+      <c r="B29" t="s">
+        <v>350</v>
+      </c>
+      <c r="C29" t="s">
+        <v>351</v>
+      </c>
+      <c r="D29">
+        <v>2025</v>
+      </c>
+      <c r="E29" t="s">
+        <v>352</v>
+      </c>
+      <c r="F29" t="s">
+        <v>353</v>
+      </c>
+      <c r="G29" t="s">
+        <v>290</v>
+      </c>
+      <c r="H29" t="s">
+        <v>12</v>
+      </c>
+      <c r="I29" t="s">
+        <v>90</v>
+      </c>
+      <c r="J29" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>355</v>
+      </c>
+      <c r="B30" t="s">
+        <v>356</v>
+      </c>
+      <c r="C30" t="s">
+        <v>233</v>
+      </c>
+      <c r="D30" t="s">
+        <v>235</v>
+      </c>
+      <c r="E30" t="s">
+        <v>304</v>
+      </c>
+      <c r="F30" t="s">
+        <v>235</v>
+      </c>
+      <c r="G30" t="s">
+        <v>290</v>
+      </c>
+      <c r="H30" t="s">
+        <v>103</v>
+      </c>
+      <c r="I30" t="s">
+        <v>357</v>
+      </c>
+      <c r="J30" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>359</v>
+      </c>
+      <c r="B31" t="s">
+        <v>360</v>
+      </c>
+      <c r="C31" t="s">
+        <v>233</v>
+      </c>
+      <c r="D31" t="s">
+        <v>361</v>
+      </c>
+      <c r="E31" t="s">
+        <v>362</v>
+      </c>
+      <c r="F31" t="s">
+        <v>235</v>
+      </c>
+      <c r="G31" t="s">
+        <v>363</v>
+      </c>
+      <c r="H31" t="s">
+        <v>103</v>
+      </c>
+      <c r="I31" t="s">
+        <v>364</v>
+      </c>
+      <c r="J31" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>366</v>
+      </c>
+      <c r="B32" t="s">
+        <v>367</v>
+      </c>
+      <c r="C32" t="s">
+        <v>233</v>
+      </c>
+      <c r="D32">
+        <v>2025</v>
+      </c>
+      <c r="E32" t="s">
+        <v>368</v>
+      </c>
+      <c r="F32" t="s">
+        <v>235</v>
+      </c>
+      <c r="G32" t="s">
+        <v>290</v>
+      </c>
+      <c r="H32" t="s">
+        <v>103</v>
+      </c>
+      <c r="I32" t="s">
+        <v>310</v>
+      </c>
+      <c r="J32" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>370</v>
+      </c>
+      <c r="B33" t="s">
+        <v>371</v>
+      </c>
+      <c r="C33" t="s">
+        <v>233</v>
+      </c>
+      <c r="D33">
+        <v>2024</v>
+      </c>
+      <c r="E33" t="s">
+        <v>372</v>
+      </c>
+      <c r="F33" t="s">
+        <v>235</v>
+      </c>
+      <c r="G33" t="s">
+        <v>290</v>
+      </c>
+      <c r="H33" t="s">
+        <v>103</v>
+      </c>
+      <c r="I33" t="s">
+        <v>373</v>
+      </c>
+      <c r="J33" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>375</v>
+      </c>
+      <c r="B34" t="s">
+        <v>376</v>
+      </c>
+      <c r="C34" t="s">
+        <v>377</v>
+      </c>
+      <c r="D34">
+        <v>2023</v>
+      </c>
+      <c r="E34" t="s">
+        <v>109</v>
+      </c>
+      <c r="F34" t="s">
+        <v>378</v>
+      </c>
+      <c r="G34" t="s">
+        <v>290</v>
+      </c>
+      <c r="H34" t="s">
+        <v>103</v>
+      </c>
+      <c r="I34" t="s">
+        <v>379</v>
+      </c>
+      <c r="J34" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>381</v>
+      </c>
+      <c r="B35" t="s">
+        <v>382</v>
+      </c>
+      <c r="C35" t="s">
+        <v>233</v>
+      </c>
+      <c r="D35">
+        <v>2025</v>
+      </c>
+      <c r="E35" t="s">
+        <v>383</v>
+      </c>
+      <c r="F35" t="s">
+        <v>235</v>
+      </c>
+      <c r="G35" t="s">
+        <v>290</v>
+      </c>
+      <c r="H35" t="s">
+        <v>103</v>
+      </c>
+      <c r="I35" t="s">
+        <v>384</v>
+      </c>
+      <c r="J35" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A36" s="10" t="s">
+        <v>418</v>
+      </c>
+      <c r="B36" s="10" t="s">
+        <v>419</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>420</v>
+      </c>
+      <c r="D36" s="10">
+        <v>2025</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>422</v>
+      </c>
+      <c r="G36" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I36" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="J36" s="10" t="s">
+        <v>424</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A37" s="10" t="s">
+        <v>425</v>
+      </c>
+      <c r="B37" s="10" t="s">
+        <v>426</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>427</v>
+      </c>
+      <c r="D37" s="10">
+        <v>2020</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>421</v>
+      </c>
+      <c r="F37" s="10" t="s">
+        <v>428</v>
+      </c>
+      <c r="G37" s="10" t="s">
+        <v>429</v>
+      </c>
+      <c r="H37" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I37" s="10" t="s">
+        <v>90</v>
+      </c>
+      <c r="J37" s="10" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="10" t="s">
+        <v>431</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>432</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D38" s="10">
+        <v>2025</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>433</v>
+      </c>
+      <c r="F38" s="10" t="s">
+        <v>434</v>
+      </c>
+      <c r="G38" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="H38" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="I38" s="10" t="s">
+        <v>435</v>
+      </c>
+      <c r="J38" s="10" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A39" s="10" t="s">
+        <v>437</v>
+      </c>
+      <c r="B39" s="10" t="s">
+        <v>438</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D39" s="10">
+        <v>2007</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>439</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="G39" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="H39" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="I39" s="10" t="s">
+        <v>440</v>
+      </c>
+      <c r="J39" s="10" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A40" s="10" t="s">
+        <v>442</v>
+      </c>
+      <c r="B40" s="10" t="s">
+        <v>443</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D40" s="10">
+        <v>2020</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>444</v>
+      </c>
+      <c r="F40" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="G40" s="10" t="s">
+        <v>445</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="I40" s="10" t="s">
+        <v>446</v>
+      </c>
+      <c r="J40" s="10" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" s="10" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A41" s="10" t="s">
+        <v>448</v>
+      </c>
+      <c r="B41" s="10" t="s">
+        <v>449</v>
+      </c>
+      <c r="C41" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="D41" s="10">
+        <v>2023</v>
+      </c>
+      <c r="E41" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="F41" s="10" t="s">
+        <v>235</v>
+      </c>
+      <c r="G41" s="10" t="s">
+        <v>423</v>
+      </c>
+      <c r="H41" s="10" t="s">
+        <v>103</v>
+      </c>
+      <c r="I41" s="10" t="s">
+        <v>451</v>
+      </c>
+      <c r="J41" s="10" t="s">
+        <v>452</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="H16:H500" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="H16:H499" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Y,N"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="G16:G500" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" sqref="G16:G499" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Pb,Cd,MB,Congo Red,Pb;Cd,MB;Congo Red"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -6108,6 +7313,2942 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{69A99B2D-2F39-4499-AAB7-FD87F89CDB32}">
+  <dimension ref="A1:T70"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="9" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="8" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="5" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="8.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="59.5546875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="122.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:19" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>285</v>
+      </c>
+      <c r="B2" t="s">
+        <v>290</v>
+      </c>
+      <c r="C2" t="s">
+        <v>323</v>
+      </c>
+      <c r="D2">
+        <v>685</v>
+      </c>
+      <c r="E2">
+        <v>0.3</v>
+      </c>
+      <c r="K2">
+        <v>6.2</v>
+      </c>
+      <c r="L2">
+        <v>1</v>
+      </c>
+      <c r="M2">
+        <v>1440</v>
+      </c>
+      <c r="N2">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P2">
+        <v>62.2</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>185</v>
+      </c>
+      <c r="R2" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B3" t="s">
+        <v>290</v>
+      </c>
+      <c r="C3" t="s">
+        <v>323</v>
+      </c>
+      <c r="D3">
+        <v>831</v>
+      </c>
+      <c r="E3">
+        <v>0.38</v>
+      </c>
+      <c r="K3">
+        <v>6.2</v>
+      </c>
+      <c r="L3">
+        <v>1</v>
+      </c>
+      <c r="M3">
+        <v>1440</v>
+      </c>
+      <c r="N3">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P3">
+        <v>137.30000000000001</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>185</v>
+      </c>
+      <c r="R3" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="4" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>285</v>
+      </c>
+      <c r="B4" t="s">
+        <v>290</v>
+      </c>
+      <c r="C4" t="s">
+        <v>323</v>
+      </c>
+      <c r="D4">
+        <v>1069</v>
+      </c>
+      <c r="E4">
+        <v>0.52</v>
+      </c>
+      <c r="K4">
+        <v>6.2</v>
+      </c>
+      <c r="L4">
+        <v>1</v>
+      </c>
+      <c r="M4">
+        <v>1440</v>
+      </c>
+      <c r="N4">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P4">
+        <v>152.9</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>185</v>
+      </c>
+      <c r="R4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>285</v>
+      </c>
+      <c r="B5" t="s">
+        <v>290</v>
+      </c>
+      <c r="C5" t="s">
+        <v>323</v>
+      </c>
+      <c r="D5">
+        <v>1669</v>
+      </c>
+      <c r="E5">
+        <v>0.91</v>
+      </c>
+      <c r="K5">
+        <v>6.2</v>
+      </c>
+      <c r="L5">
+        <v>1</v>
+      </c>
+      <c r="M5">
+        <v>1440</v>
+      </c>
+      <c r="N5">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P5">
+        <v>444</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>185</v>
+      </c>
+      <c r="R5" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="6" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>292</v>
+      </c>
+      <c r="B6" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" t="s">
+        <v>325</v>
+      </c>
+      <c r="D6">
+        <v>348.00170000000003</v>
+      </c>
+      <c r="E6">
+        <v>0.15351799999999999</v>
+      </c>
+      <c r="F6">
+        <v>6.03</v>
+      </c>
+      <c r="G6">
+        <v>82.08</v>
+      </c>
+      <c r="I6">
+        <v>15.09</v>
+      </c>
+      <c r="L6">
+        <v>7</v>
+      </c>
+      <c r="M6">
+        <v>2.5</v>
+      </c>
+      <c r="N6">
+        <v>90</v>
+      </c>
+      <c r="O6">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q6">
+        <v>57.47</v>
+      </c>
+      <c r="R6" t="s">
+        <v>185</v>
+      </c>
+      <c r="S6" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="7" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>292</v>
+      </c>
+      <c r="B7" t="s">
+        <v>290</v>
+      </c>
+      <c r="C7" t="s">
+        <v>325</v>
+      </c>
+      <c r="D7">
+        <v>348.00170000000003</v>
+      </c>
+      <c r="E7">
+        <v>0.15351799999999999</v>
+      </c>
+      <c r="F7">
+        <v>6.03</v>
+      </c>
+      <c r="G7">
+        <v>82.08</v>
+      </c>
+      <c r="I7">
+        <v>15.09</v>
+      </c>
+      <c r="K7">
+        <v>54.91</v>
+      </c>
+      <c r="L7">
+        <v>7</v>
+      </c>
+      <c r="M7">
+        <v>2.5</v>
+      </c>
+      <c r="N7">
+        <v>60</v>
+      </c>
+      <c r="O7">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q7">
+        <v>20.89</v>
+      </c>
+      <c r="R7" t="s">
+        <v>185</v>
+      </c>
+      <c r="S7" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>292</v>
+      </c>
+      <c r="B8" t="s">
+        <v>290</v>
+      </c>
+      <c r="C8" t="s">
+        <v>325</v>
+      </c>
+      <c r="D8">
+        <v>348.00170000000003</v>
+      </c>
+      <c r="E8">
+        <v>0.15351799999999999</v>
+      </c>
+      <c r="F8">
+        <v>6.03</v>
+      </c>
+      <c r="G8">
+        <v>82.08</v>
+      </c>
+      <c r="I8">
+        <v>15.09</v>
+      </c>
+      <c r="K8">
+        <v>84.65</v>
+      </c>
+      <c r="L8">
+        <v>7</v>
+      </c>
+      <c r="M8">
+        <v>2.5</v>
+      </c>
+      <c r="N8">
+        <v>60</v>
+      </c>
+      <c r="O8">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q8">
+        <v>30.57</v>
+      </c>
+      <c r="R8" t="s">
+        <v>185</v>
+      </c>
+      <c r="S8" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>292</v>
+      </c>
+      <c r="B9" t="s">
+        <v>290</v>
+      </c>
+      <c r="C9" t="s">
+        <v>325</v>
+      </c>
+      <c r="D9">
+        <v>348.00170000000003</v>
+      </c>
+      <c r="E9">
+        <v>0.15351799999999999</v>
+      </c>
+      <c r="F9">
+        <v>6.03</v>
+      </c>
+      <c r="G9">
+        <v>82.08</v>
+      </c>
+      <c r="I9">
+        <v>15.09</v>
+      </c>
+      <c r="K9">
+        <v>112.4</v>
+      </c>
+      <c r="L9">
+        <v>7</v>
+      </c>
+      <c r="M9">
+        <v>2.5</v>
+      </c>
+      <c r="N9">
+        <v>60</v>
+      </c>
+      <c r="O9">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q9">
+        <v>32.6</v>
+      </c>
+      <c r="R9" t="s">
+        <v>185</v>
+      </c>
+      <c r="S9" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>297</v>
+      </c>
+      <c r="B10" t="s">
+        <v>290</v>
+      </c>
+      <c r="C10" t="s">
+        <v>328</v>
+      </c>
+      <c r="D10">
+        <v>339.6</v>
+      </c>
+      <c r="E10">
+        <v>0.16</v>
+      </c>
+      <c r="F10">
+        <v>7.7</v>
+      </c>
+      <c r="G10">
+        <v>90.48</v>
+      </c>
+      <c r="I10">
+        <v>3.81</v>
+      </c>
+      <c r="J10">
+        <v>2.2400000000000002</v>
+      </c>
+      <c r="L10">
+        <v>2</v>
+      </c>
+      <c r="M10">
+        <v>3000</v>
+      </c>
+      <c r="N10">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P10">
+        <v>199.7</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>185</v>
+      </c>
+      <c r="R10" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>297</v>
+      </c>
+      <c r="B11" t="s">
+        <v>290</v>
+      </c>
+      <c r="C11" t="s">
+        <v>328</v>
+      </c>
+      <c r="D11">
+        <v>358.4</v>
+      </c>
+      <c r="E11">
+        <v>0.17899999999999999</v>
+      </c>
+      <c r="F11">
+        <v>7.5</v>
+      </c>
+      <c r="L11">
+        <v>2</v>
+      </c>
+      <c r="M11">
+        <v>3000</v>
+      </c>
+      <c r="N11">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P11">
+        <v>193.74</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>185</v>
+      </c>
+      <c r="R11" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>297</v>
+      </c>
+      <c r="B12" t="s">
+        <v>290</v>
+      </c>
+      <c r="C12" t="s">
+        <v>328</v>
+      </c>
+      <c r="D12">
+        <v>594</v>
+      </c>
+      <c r="E12">
+        <v>0.35599999999999998</v>
+      </c>
+      <c r="F12">
+        <v>8.4</v>
+      </c>
+      <c r="G12">
+        <v>73.03</v>
+      </c>
+      <c r="I12">
+        <v>11.28</v>
+      </c>
+      <c r="J12">
+        <v>1.22</v>
+      </c>
+      <c r="L12">
+        <v>2</v>
+      </c>
+      <c r="M12">
+        <v>3000</v>
+      </c>
+      <c r="N12">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P12">
+        <v>194.99</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>185</v>
+      </c>
+      <c r="R12" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>297</v>
+      </c>
+      <c r="B13" t="s">
+        <v>290</v>
+      </c>
+      <c r="C13" t="s">
+        <v>328</v>
+      </c>
+      <c r="D13">
+        <v>600.4</v>
+      </c>
+      <c r="E13">
+        <v>0.38</v>
+      </c>
+      <c r="F13">
+        <v>7.6</v>
+      </c>
+      <c r="G13">
+        <v>83.89</v>
+      </c>
+      <c r="I13">
+        <v>6.13</v>
+      </c>
+      <c r="J13">
+        <v>1.92</v>
+      </c>
+      <c r="L13">
+        <v>2</v>
+      </c>
+      <c r="M13">
+        <v>3000</v>
+      </c>
+      <c r="N13">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P13">
+        <v>225.31</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>185</v>
+      </c>
+      <c r="R13" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>297</v>
+      </c>
+      <c r="B14" t="s">
+        <v>290</v>
+      </c>
+      <c r="C14" t="s">
+        <v>328</v>
+      </c>
+      <c r="D14">
+        <v>346.7</v>
+      </c>
+      <c r="E14">
+        <v>0.157</v>
+      </c>
+      <c r="F14">
+        <v>8.4</v>
+      </c>
+      <c r="G14">
+        <v>86.57</v>
+      </c>
+      <c r="I14">
+        <v>7.08</v>
+      </c>
+      <c r="J14">
+        <v>2.69</v>
+      </c>
+      <c r="L14">
+        <v>2</v>
+      </c>
+      <c r="M14">
+        <v>3000</v>
+      </c>
+      <c r="N14">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P14">
+        <v>194.18</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>185</v>
+      </c>
+      <c r="R14" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>297</v>
+      </c>
+      <c r="B15" t="s">
+        <v>290</v>
+      </c>
+      <c r="C15" t="s">
+        <v>328</v>
+      </c>
+      <c r="D15">
+        <v>393.9</v>
+      </c>
+      <c r="E15">
+        <v>0.19700000000000001</v>
+      </c>
+      <c r="F15">
+        <v>7.6</v>
+      </c>
+      <c r="L15">
+        <v>2</v>
+      </c>
+      <c r="M15">
+        <v>3000</v>
+      </c>
+      <c r="N15">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P15">
+        <v>200.01</v>
+      </c>
+      <c r="Q15" t="s">
+        <v>185</v>
+      </c>
+      <c r="R15" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="16" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>302</v>
+      </c>
+      <c r="B16" t="s">
+        <v>290</v>
+      </c>
+      <c r="C16" t="s">
+        <v>335</v>
+      </c>
+      <c r="D16">
+        <v>1530.67</v>
+      </c>
+      <c r="E16">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F16">
+        <v>6.3</v>
+      </c>
+      <c r="K16">
+        <v>150</v>
+      </c>
+      <c r="L16">
+        <v>7.5</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+      <c r="N16">
+        <v>180</v>
+      </c>
+      <c r="O16">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q16">
+        <v>149.9</v>
+      </c>
+      <c r="R16" t="s">
+        <v>185</v>
+      </c>
+      <c r="S16" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>302</v>
+      </c>
+      <c r="B17" t="s">
+        <v>290</v>
+      </c>
+      <c r="C17" t="s">
+        <v>335</v>
+      </c>
+      <c r="D17">
+        <v>1530.67</v>
+      </c>
+      <c r="E17">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F17">
+        <v>6.3</v>
+      </c>
+      <c r="K17">
+        <v>200</v>
+      </c>
+      <c r="L17">
+        <v>7.5</v>
+      </c>
+      <c r="M17">
+        <v>1</v>
+      </c>
+      <c r="N17">
+        <v>180</v>
+      </c>
+      <c r="O17">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q17">
+        <v>199.7</v>
+      </c>
+      <c r="R17" t="s">
+        <v>185</v>
+      </c>
+      <c r="S17" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>302</v>
+      </c>
+      <c r="B18" t="s">
+        <v>290</v>
+      </c>
+      <c r="C18" t="s">
+        <v>335</v>
+      </c>
+      <c r="D18">
+        <v>1530.67</v>
+      </c>
+      <c r="E18">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F18">
+        <v>6.3</v>
+      </c>
+      <c r="K18">
+        <v>250</v>
+      </c>
+      <c r="L18">
+        <v>7.5</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
+      </c>
+      <c r="N18">
+        <v>180</v>
+      </c>
+      <c r="O18">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q18">
+        <v>248.8</v>
+      </c>
+      <c r="R18" t="s">
+        <v>185</v>
+      </c>
+      <c r="S18" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>302</v>
+      </c>
+      <c r="B19" t="s">
+        <v>290</v>
+      </c>
+      <c r="C19" t="s">
+        <v>335</v>
+      </c>
+      <c r="D19">
+        <v>1530.67</v>
+      </c>
+      <c r="E19">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F19">
+        <v>6.3</v>
+      </c>
+      <c r="M19">
+        <v>180</v>
+      </c>
+      <c r="N19">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P19">
+        <v>324.7</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>185</v>
+      </c>
+      <c r="R19" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>307</v>
+      </c>
+      <c r="B20" t="s">
+        <v>290</v>
+      </c>
+      <c r="C20" t="s">
+        <v>338</v>
+      </c>
+      <c r="D20">
+        <v>678.8</v>
+      </c>
+      <c r="E20">
+        <v>0.34200000000000003</v>
+      </c>
+      <c r="K20">
+        <v>100</v>
+      </c>
+      <c r="L20">
+        <v>7</v>
+      </c>
+      <c r="M20">
+        <v>0.5</v>
+      </c>
+      <c r="N20">
+        <v>100</v>
+      </c>
+      <c r="O20">
+        <v>300.14999999999998</v>
+      </c>
+      <c r="Q20">
+        <v>93</v>
+      </c>
+      <c r="R20" t="s">
+        <v>200</v>
+      </c>
+      <c r="S20" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>312</v>
+      </c>
+      <c r="B21" t="s">
+        <v>290</v>
+      </c>
+      <c r="C21" t="s">
+        <v>340</v>
+      </c>
+      <c r="D21">
+        <v>932</v>
+      </c>
+      <c r="E21">
+        <v>0.437</v>
+      </c>
+      <c r="F21">
+        <v>8.77</v>
+      </c>
+      <c r="N21">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="P21">
+        <v>459.35</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>185</v>
+      </c>
+      <c r="R21" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>312</v>
+      </c>
+      <c r="B22" t="s">
+        <v>290</v>
+      </c>
+      <c r="C22" t="s">
+        <v>340</v>
+      </c>
+      <c r="D22">
+        <v>926</v>
+      </c>
+      <c r="E22">
+        <v>0.442</v>
+      </c>
+      <c r="F22">
+        <v>8.81</v>
+      </c>
+      <c r="N22">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="P22">
+        <v>497.12</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>185</v>
+      </c>
+      <c r="R22" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="23" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>312</v>
+      </c>
+      <c r="B23" t="s">
+        <v>290</v>
+      </c>
+      <c r="C23" t="s">
+        <v>340</v>
+      </c>
+      <c r="D23">
+        <v>1140</v>
+      </c>
+      <c r="E23">
+        <v>0.58699999999999997</v>
+      </c>
+      <c r="F23">
+        <v>9.48</v>
+      </c>
+      <c r="N23">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="P23">
+        <v>648.12</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>185</v>
+      </c>
+      <c r="R23" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="24" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>312</v>
+      </c>
+      <c r="B24" t="s">
+        <v>290</v>
+      </c>
+      <c r="C24" t="s">
+        <v>340</v>
+      </c>
+      <c r="D24">
+        <v>980</v>
+      </c>
+      <c r="E24">
+        <v>0.48</v>
+      </c>
+      <c r="F24">
+        <v>9.36</v>
+      </c>
+      <c r="N24">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="P24">
+        <v>488.29</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>185</v>
+      </c>
+      <c r="R24" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="25" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>312</v>
+      </c>
+      <c r="B25" t="s">
+        <v>290</v>
+      </c>
+      <c r="C25" t="s">
+        <v>340</v>
+      </c>
+      <c r="D25">
+        <v>1271</v>
+      </c>
+      <c r="E25">
+        <v>0.73599999999999999</v>
+      </c>
+      <c r="F25">
+        <v>9.5399999999999991</v>
+      </c>
+      <c r="N25">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="P25">
+        <v>714.29</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>185</v>
+      </c>
+      <c r="R25" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="26" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>312</v>
+      </c>
+      <c r="B26" t="s">
+        <v>290</v>
+      </c>
+      <c r="C26" t="s">
+        <v>340</v>
+      </c>
+      <c r="D26">
+        <v>1773</v>
+      </c>
+      <c r="E26">
+        <v>1.0740000000000001</v>
+      </c>
+      <c r="F26">
+        <v>9.94</v>
+      </c>
+      <c r="N26">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="P26">
+        <v>1000</v>
+      </c>
+      <c r="Q26" t="s">
+        <v>185</v>
+      </c>
+      <c r="R26" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="27" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>317</v>
+      </c>
+      <c r="B27" t="s">
+        <v>290</v>
+      </c>
+      <c r="C27" t="s">
+        <v>347</v>
+      </c>
+      <c r="D27">
+        <v>1540</v>
+      </c>
+      <c r="E27">
+        <v>0.67369999999999997</v>
+      </c>
+      <c r="K27">
+        <v>100.9</v>
+      </c>
+      <c r="L27">
+        <v>10.199999999999999</v>
+      </c>
+      <c r="M27">
+        <v>0.69399999999999995</v>
+      </c>
+      <c r="N27">
+        <v>149.1</v>
+      </c>
+      <c r="O27">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q27">
+        <v>571.70000000000005</v>
+      </c>
+      <c r="R27" t="s">
+        <v>185</v>
+      </c>
+      <c r="S27" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>349</v>
+      </c>
+      <c r="B28" t="s">
+        <v>290</v>
+      </c>
+      <c r="C28" t="s">
+        <v>386</v>
+      </c>
+      <c r="D28">
+        <v>808</v>
+      </c>
+      <c r="E28">
+        <v>0.37</v>
+      </c>
+      <c r="F28">
+        <v>5.6</v>
+      </c>
+      <c r="K28">
+        <v>50</v>
+      </c>
+      <c r="L28">
+        <v>7</v>
+      </c>
+      <c r="M28">
+        <v>4</v>
+      </c>
+      <c r="N28">
+        <v>60</v>
+      </c>
+      <c r="O28">
+        <v>298</v>
+      </c>
+      <c r="Q28">
+        <v>46.1</v>
+      </c>
+      <c r="R28" t="s">
+        <v>185</v>
+      </c>
+      <c r="S28" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="29" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>349</v>
+      </c>
+      <c r="B29" t="s">
+        <v>290</v>
+      </c>
+      <c r="C29" t="s">
+        <v>386</v>
+      </c>
+      <c r="D29">
+        <v>749</v>
+      </c>
+      <c r="E29">
+        <v>0.68</v>
+      </c>
+      <c r="F29">
+        <v>4.96</v>
+      </c>
+      <c r="K29">
+        <v>50</v>
+      </c>
+      <c r="L29">
+        <v>7</v>
+      </c>
+      <c r="M29">
+        <v>4</v>
+      </c>
+      <c r="N29">
+        <v>60</v>
+      </c>
+      <c r="O29">
+        <v>298</v>
+      </c>
+      <c r="Q29">
+        <v>57.8</v>
+      </c>
+      <c r="R29" t="s">
+        <v>185</v>
+      </c>
+      <c r="S29" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>349</v>
+      </c>
+      <c r="B30" t="s">
+        <v>290</v>
+      </c>
+      <c r="C30" t="s">
+        <v>386</v>
+      </c>
+      <c r="D30">
+        <v>731</v>
+      </c>
+      <c r="E30">
+        <v>0.78</v>
+      </c>
+      <c r="F30">
+        <v>5.38</v>
+      </c>
+      <c r="K30">
+        <v>50</v>
+      </c>
+      <c r="L30">
+        <v>7</v>
+      </c>
+      <c r="M30">
+        <v>4</v>
+      </c>
+      <c r="N30">
+        <v>60</v>
+      </c>
+      <c r="O30">
+        <v>298</v>
+      </c>
+      <c r="Q30">
+        <v>58.5</v>
+      </c>
+      <c r="R30" t="s">
+        <v>185</v>
+      </c>
+      <c r="S30" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>349</v>
+      </c>
+      <c r="B31" t="s">
+        <v>290</v>
+      </c>
+      <c r="C31" t="s">
+        <v>386</v>
+      </c>
+      <c r="D31">
+        <v>724</v>
+      </c>
+      <c r="E31">
+        <v>0.66</v>
+      </c>
+      <c r="F31">
+        <v>5.15</v>
+      </c>
+      <c r="K31">
+        <v>50</v>
+      </c>
+      <c r="L31">
+        <v>7</v>
+      </c>
+      <c r="M31">
+        <v>4</v>
+      </c>
+      <c r="N31">
+        <v>60</v>
+      </c>
+      <c r="O31">
+        <v>298</v>
+      </c>
+      <c r="Q31">
+        <v>53.5</v>
+      </c>
+      <c r="R31" t="s">
+        <v>185</v>
+      </c>
+      <c r="S31" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>349</v>
+      </c>
+      <c r="B32" t="s">
+        <v>290</v>
+      </c>
+      <c r="C32" t="s">
+        <v>386</v>
+      </c>
+      <c r="D32">
+        <v>808</v>
+      </c>
+      <c r="E32">
+        <v>0.37</v>
+      </c>
+      <c r="F32">
+        <v>5.6</v>
+      </c>
+      <c r="L32">
+        <v>7</v>
+      </c>
+      <c r="M32">
+        <v>4</v>
+      </c>
+      <c r="O32">
+        <v>298</v>
+      </c>
+      <c r="Q32">
+        <v>30.2</v>
+      </c>
+      <c r="R32" t="s">
+        <v>185</v>
+      </c>
+      <c r="S32" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="33" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>349</v>
+      </c>
+      <c r="B33" t="s">
+        <v>290</v>
+      </c>
+      <c r="C33" t="s">
+        <v>386</v>
+      </c>
+      <c r="D33">
+        <v>749</v>
+      </c>
+      <c r="E33">
+        <v>0.68</v>
+      </c>
+      <c r="F33">
+        <v>4.96</v>
+      </c>
+      <c r="L33">
+        <v>7</v>
+      </c>
+      <c r="M33">
+        <v>4</v>
+      </c>
+      <c r="O33">
+        <v>298</v>
+      </c>
+      <c r="Q33">
+        <v>52.6</v>
+      </c>
+      <c r="R33" t="s">
+        <v>185</v>
+      </c>
+      <c r="S33" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="34" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>349</v>
+      </c>
+      <c r="B34" t="s">
+        <v>290</v>
+      </c>
+      <c r="C34" t="s">
+        <v>386</v>
+      </c>
+      <c r="D34">
+        <v>731</v>
+      </c>
+      <c r="E34">
+        <v>0.78</v>
+      </c>
+      <c r="F34">
+        <v>5.38</v>
+      </c>
+      <c r="L34">
+        <v>7</v>
+      </c>
+      <c r="M34">
+        <v>4</v>
+      </c>
+      <c r="O34">
+        <v>298</v>
+      </c>
+      <c r="Q34">
+        <v>31.1</v>
+      </c>
+      <c r="R34" t="s">
+        <v>185</v>
+      </c>
+      <c r="S34" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="35" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>349</v>
+      </c>
+      <c r="B35" t="s">
+        <v>290</v>
+      </c>
+      <c r="C35" t="s">
+        <v>386</v>
+      </c>
+      <c r="D35">
+        <v>724</v>
+      </c>
+      <c r="E35">
+        <v>0.66</v>
+      </c>
+      <c r="F35">
+        <v>5.15</v>
+      </c>
+      <c r="L35">
+        <v>7</v>
+      </c>
+      <c r="M35">
+        <v>4</v>
+      </c>
+      <c r="O35">
+        <v>298</v>
+      </c>
+      <c r="Q35">
+        <v>36.4</v>
+      </c>
+      <c r="R35" t="s">
+        <v>185</v>
+      </c>
+      <c r="S35" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>355</v>
+      </c>
+      <c r="B36" t="s">
+        <v>290</v>
+      </c>
+      <c r="C36" t="s">
+        <v>335</v>
+      </c>
+      <c r="D36">
+        <v>1530.67</v>
+      </c>
+      <c r="E36">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F36">
+        <v>6.3</v>
+      </c>
+      <c r="M36">
+        <v>180</v>
+      </c>
+      <c r="N36">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P36">
+        <v>324.7</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>185</v>
+      </c>
+      <c r="R36" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="37" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>355</v>
+      </c>
+      <c r="B37" t="s">
+        <v>290</v>
+      </c>
+      <c r="C37" t="s">
+        <v>335</v>
+      </c>
+      <c r="D37">
+        <v>1530.67</v>
+      </c>
+      <c r="E37">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F37">
+        <v>6.3</v>
+      </c>
+      <c r="K37">
+        <v>150</v>
+      </c>
+      <c r="L37">
+        <v>7.5</v>
+      </c>
+      <c r="M37">
+        <v>1</v>
+      </c>
+      <c r="N37">
+        <v>180</v>
+      </c>
+      <c r="O37">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q37">
+        <v>149.9</v>
+      </c>
+      <c r="R37" t="s">
+        <v>185</v>
+      </c>
+      <c r="S37" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>355</v>
+      </c>
+      <c r="B38" t="s">
+        <v>290</v>
+      </c>
+      <c r="C38" t="s">
+        <v>335</v>
+      </c>
+      <c r="D38">
+        <v>1530.67</v>
+      </c>
+      <c r="E38">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F38">
+        <v>6.3</v>
+      </c>
+      <c r="K38">
+        <v>200</v>
+      </c>
+      <c r="L38">
+        <v>7.5</v>
+      </c>
+      <c r="M38">
+        <v>1</v>
+      </c>
+      <c r="N38">
+        <v>180</v>
+      </c>
+      <c r="O38">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q38">
+        <v>199.7</v>
+      </c>
+      <c r="R38" t="s">
+        <v>185</v>
+      </c>
+      <c r="S38" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="39" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>355</v>
+      </c>
+      <c r="B39" t="s">
+        <v>290</v>
+      </c>
+      <c r="C39" t="s">
+        <v>335</v>
+      </c>
+      <c r="D39">
+        <v>1530.67</v>
+      </c>
+      <c r="E39">
+        <v>0.78259999999999996</v>
+      </c>
+      <c r="F39">
+        <v>6.3</v>
+      </c>
+      <c r="K39">
+        <v>250</v>
+      </c>
+      <c r="L39">
+        <v>7.5</v>
+      </c>
+      <c r="M39">
+        <v>1</v>
+      </c>
+      <c r="N39">
+        <v>180</v>
+      </c>
+      <c r="O39">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q39">
+        <v>248.8</v>
+      </c>
+      <c r="R39" t="s">
+        <v>185</v>
+      </c>
+      <c r="S39" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A40" t="s">
+        <v>359</v>
+      </c>
+      <c r="B40" t="s">
+        <v>290</v>
+      </c>
+      <c r="C40" t="s">
+        <v>397</v>
+      </c>
+      <c r="D40">
+        <v>1902.3</v>
+      </c>
+      <c r="E40">
+        <v>0.88</v>
+      </c>
+      <c r="F40">
+        <v>6.58</v>
+      </c>
+      <c r="G40">
+        <v>73.39</v>
+      </c>
+      <c r="H40">
+        <v>4.16</v>
+      </c>
+      <c r="I40">
+        <v>21.75</v>
+      </c>
+      <c r="J40">
+        <v>0.71</v>
+      </c>
+      <c r="L40">
+        <v>7</v>
+      </c>
+      <c r="M40">
+        <v>0.5</v>
+      </c>
+      <c r="O40">
+        <v>303.14999999999998</v>
+      </c>
+      <c r="Q40">
+        <v>838.42</v>
+      </c>
+      <c r="R40" t="s">
+        <v>185</v>
+      </c>
+      <c r="S40" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="41" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A41" t="s">
+        <v>359</v>
+      </c>
+      <c r="B41" t="s">
+        <v>290</v>
+      </c>
+      <c r="C41" t="s">
+        <v>399</v>
+      </c>
+      <c r="D41">
+        <v>1115.9000000000001</v>
+      </c>
+      <c r="E41">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="F41">
+        <v>6.47</v>
+      </c>
+      <c r="G41">
+        <v>54.79</v>
+      </c>
+      <c r="H41">
+        <v>2.84</v>
+      </c>
+      <c r="I41">
+        <v>41.62</v>
+      </c>
+      <c r="J41">
+        <v>0.76</v>
+      </c>
+      <c r="L41">
+        <v>7</v>
+      </c>
+      <c r="M41">
+        <v>0.5</v>
+      </c>
+      <c r="O41">
+        <v>303.14999999999998</v>
+      </c>
+      <c r="Q41">
+        <v>855.96</v>
+      </c>
+      <c r="R41" t="s">
+        <v>185</v>
+      </c>
+      <c r="S41" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>359</v>
+      </c>
+      <c r="B42" t="s">
+        <v>290</v>
+      </c>
+      <c r="C42" t="s">
+        <v>401</v>
+      </c>
+      <c r="D42">
+        <v>1412.4</v>
+      </c>
+      <c r="E42">
+        <v>0.66</v>
+      </c>
+      <c r="F42">
+        <v>6.42</v>
+      </c>
+      <c r="G42">
+        <v>69.7</v>
+      </c>
+      <c r="H42">
+        <v>3.09</v>
+      </c>
+      <c r="I42">
+        <v>26.59</v>
+      </c>
+      <c r="J42">
+        <v>0.62</v>
+      </c>
+      <c r="L42">
+        <v>7</v>
+      </c>
+      <c r="M42">
+        <v>0.5</v>
+      </c>
+      <c r="O42">
+        <v>303.14999999999998</v>
+      </c>
+      <c r="Q42">
+        <v>826.28</v>
+      </c>
+      <c r="R42" t="s">
+        <v>185</v>
+      </c>
+      <c r="S42" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A43" t="s">
+        <v>359</v>
+      </c>
+      <c r="B43" t="s">
+        <v>290</v>
+      </c>
+      <c r="C43" t="s">
+        <v>397</v>
+      </c>
+      <c r="D43">
+        <v>1902.3</v>
+      </c>
+      <c r="E43">
+        <v>0.88</v>
+      </c>
+      <c r="F43">
+        <v>6.58</v>
+      </c>
+      <c r="G43">
+        <v>73.39</v>
+      </c>
+      <c r="H43">
+        <v>4.16</v>
+      </c>
+      <c r="I43">
+        <v>21.75</v>
+      </c>
+      <c r="J43">
+        <v>0.71</v>
+      </c>
+      <c r="K43">
+        <v>300</v>
+      </c>
+      <c r="L43">
+        <v>7</v>
+      </c>
+      <c r="M43">
+        <v>0.5</v>
+      </c>
+      <c r="N43">
+        <v>120</v>
+      </c>
+      <c r="O43">
+        <v>303.14999999999998</v>
+      </c>
+      <c r="Q43">
+        <v>509.47</v>
+      </c>
+      <c r="R43" t="s">
+        <v>185</v>
+      </c>
+      <c r="S43" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="44" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A44" t="s">
+        <v>359</v>
+      </c>
+      <c r="B44" t="s">
+        <v>290</v>
+      </c>
+      <c r="C44" t="s">
+        <v>399</v>
+      </c>
+      <c r="D44">
+        <v>1115.9000000000001</v>
+      </c>
+      <c r="E44">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="F44">
+        <v>6.47</v>
+      </c>
+      <c r="G44">
+        <v>54.79</v>
+      </c>
+      <c r="H44">
+        <v>2.84</v>
+      </c>
+      <c r="I44">
+        <v>41.62</v>
+      </c>
+      <c r="J44">
+        <v>0.76</v>
+      </c>
+      <c r="K44">
+        <v>300</v>
+      </c>
+      <c r="L44">
+        <v>7</v>
+      </c>
+      <c r="M44">
+        <v>0.5</v>
+      </c>
+      <c r="N44">
+        <v>120</v>
+      </c>
+      <c r="O44">
+        <v>303.14999999999998</v>
+      </c>
+      <c r="Q44">
+        <v>458.9</v>
+      </c>
+      <c r="R44" t="s">
+        <v>185</v>
+      </c>
+      <c r="S44" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="45" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A45" t="s">
+        <v>359</v>
+      </c>
+      <c r="B45" t="s">
+        <v>290</v>
+      </c>
+      <c r="C45" t="s">
+        <v>401</v>
+      </c>
+      <c r="D45">
+        <v>1412.4</v>
+      </c>
+      <c r="E45">
+        <v>0.66</v>
+      </c>
+      <c r="F45">
+        <v>6.42</v>
+      </c>
+      <c r="G45">
+        <v>69.7</v>
+      </c>
+      <c r="H45">
+        <v>3.09</v>
+      </c>
+      <c r="I45">
+        <v>26.59</v>
+      </c>
+      <c r="J45">
+        <v>0.62</v>
+      </c>
+      <c r="K45">
+        <v>300</v>
+      </c>
+      <c r="L45">
+        <v>7</v>
+      </c>
+      <c r="M45">
+        <v>0.5</v>
+      </c>
+      <c r="N45">
+        <v>120</v>
+      </c>
+      <c r="O45">
+        <v>303.14999999999998</v>
+      </c>
+      <c r="Q45">
+        <v>478.36</v>
+      </c>
+      <c r="R45" t="s">
+        <v>185</v>
+      </c>
+      <c r="S45" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A46" t="s">
+        <v>366</v>
+      </c>
+      <c r="B46" t="s">
+        <v>290</v>
+      </c>
+      <c r="C46" t="s">
+        <v>406</v>
+      </c>
+      <c r="D46">
+        <v>1565</v>
+      </c>
+      <c r="E46">
+        <v>0.67600000000000005</v>
+      </c>
+      <c r="L46">
+        <v>4</v>
+      </c>
+      <c r="M46">
+        <v>180</v>
+      </c>
+      <c r="N46">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P46">
+        <v>34.299999999999997</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>185</v>
+      </c>
+      <c r="R46" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="47" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A47" t="s">
+        <v>366</v>
+      </c>
+      <c r="B47" t="s">
+        <v>290</v>
+      </c>
+      <c r="C47" t="s">
+        <v>406</v>
+      </c>
+      <c r="D47">
+        <v>1565</v>
+      </c>
+      <c r="E47">
+        <v>0.67600000000000005</v>
+      </c>
+      <c r="L47">
+        <v>4</v>
+      </c>
+      <c r="N47">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P47">
+        <v>235.21</v>
+      </c>
+      <c r="Q47" t="s">
+        <v>185</v>
+      </c>
+      <c r="R47" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="48" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>366</v>
+      </c>
+      <c r="B48" t="s">
+        <v>290</v>
+      </c>
+      <c r="C48" t="s">
+        <v>406</v>
+      </c>
+      <c r="D48">
+        <v>1565</v>
+      </c>
+      <c r="E48">
+        <v>0.67600000000000005</v>
+      </c>
+      <c r="L48">
+        <v>4</v>
+      </c>
+      <c r="N48">
+        <v>303.14999999999998</v>
+      </c>
+      <c r="P48">
+        <v>209.62</v>
+      </c>
+      <c r="Q48" t="s">
+        <v>185</v>
+      </c>
+      <c r="R48" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A49" t="s">
+        <v>366</v>
+      </c>
+      <c r="B49" t="s">
+        <v>290</v>
+      </c>
+      <c r="C49" t="s">
+        <v>406</v>
+      </c>
+      <c r="D49">
+        <v>1565</v>
+      </c>
+      <c r="E49">
+        <v>0.67600000000000005</v>
+      </c>
+      <c r="L49">
+        <v>4</v>
+      </c>
+      <c r="N49">
+        <v>313.14999999999998</v>
+      </c>
+      <c r="P49">
+        <v>198.62</v>
+      </c>
+      <c r="Q49" t="s">
+        <v>185</v>
+      </c>
+      <c r="R49" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A50" t="s">
+        <v>366</v>
+      </c>
+      <c r="B50" t="s">
+        <v>290</v>
+      </c>
+      <c r="C50" t="s">
+        <v>406</v>
+      </c>
+      <c r="D50">
+        <v>1565</v>
+      </c>
+      <c r="E50">
+        <v>0.67600000000000005</v>
+      </c>
+      <c r="J50">
+        <v>100</v>
+      </c>
+      <c r="L50">
+        <v>4</v>
+      </c>
+      <c r="M50">
+        <v>180</v>
+      </c>
+      <c r="N50">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="P50">
+        <v>23.21</v>
+      </c>
+      <c r="Q50" t="s">
+        <v>185</v>
+      </c>
+      <c r="R50" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A51" t="s">
+        <v>375</v>
+      </c>
+      <c r="B51" t="s">
+        <v>290</v>
+      </c>
+      <c r="C51" t="s">
+        <v>410</v>
+      </c>
+      <c r="D51">
+        <v>282.02</v>
+      </c>
+      <c r="E51">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="F51">
+        <v>7.5</v>
+      </c>
+      <c r="L51">
+        <v>500</v>
+      </c>
+      <c r="N51">
+        <v>0.3</v>
+      </c>
+      <c r="O51">
+        <v>180</v>
+      </c>
+      <c r="P51">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="R51">
+        <v>384</v>
+      </c>
+      <c r="S51" t="s">
+        <v>185</v>
+      </c>
+      <c r="T51" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A52" t="s">
+        <v>375</v>
+      </c>
+      <c r="B52" t="s">
+        <v>290</v>
+      </c>
+      <c r="C52" t="s">
+        <v>410</v>
+      </c>
+      <c r="D52">
+        <v>282.02</v>
+      </c>
+      <c r="E52">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="F52">
+        <v>7.5</v>
+      </c>
+      <c r="M52">
+        <v>0.2</v>
+      </c>
+      <c r="N52">
+        <v>180</v>
+      </c>
+      <c r="O52">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q52">
+        <v>469</v>
+      </c>
+      <c r="R52" t="s">
+        <v>412</v>
+      </c>
+      <c r="S52" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>375</v>
+      </c>
+      <c r="B53" t="s">
+        <v>290</v>
+      </c>
+      <c r="C53" t="s">
+        <v>410</v>
+      </c>
+      <c r="D53">
+        <v>282.02</v>
+      </c>
+      <c r="E53">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="F53">
+        <v>7.5</v>
+      </c>
+      <c r="L53">
+        <v>500</v>
+      </c>
+      <c r="N53">
+        <v>0.3</v>
+      </c>
+      <c r="O53">
+        <v>180</v>
+      </c>
+      <c r="P53">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="R53">
+        <v>387</v>
+      </c>
+      <c r="S53" t="s">
+        <v>185</v>
+      </c>
+      <c r="T53" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A54" t="s">
+        <v>375</v>
+      </c>
+      <c r="B54" t="s">
+        <v>290</v>
+      </c>
+      <c r="C54" t="s">
+        <v>410</v>
+      </c>
+      <c r="D54">
+        <v>282.02</v>
+      </c>
+      <c r="E54">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="F54">
+        <v>7.5</v>
+      </c>
+      <c r="L54">
+        <v>500</v>
+      </c>
+      <c r="N54">
+        <v>0.3</v>
+      </c>
+      <c r="O54">
+        <v>180</v>
+      </c>
+      <c r="P54">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="R54">
+        <v>528</v>
+      </c>
+      <c r="S54" t="s">
+        <v>185</v>
+      </c>
+      <c r="T54" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>375</v>
+      </c>
+      <c r="B55" t="s">
+        <v>290</v>
+      </c>
+      <c r="C55" t="s">
+        <v>410</v>
+      </c>
+      <c r="D55">
+        <v>282.02</v>
+      </c>
+      <c r="E55">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="F55">
+        <v>7.5</v>
+      </c>
+      <c r="L55">
+        <v>500</v>
+      </c>
+      <c r="N55">
+        <v>0.3</v>
+      </c>
+      <c r="O55">
+        <v>180</v>
+      </c>
+      <c r="P55">
+        <v>318.14999999999998</v>
+      </c>
+      <c r="R55">
+        <v>835</v>
+      </c>
+      <c r="S55" t="s">
+        <v>185</v>
+      </c>
+      <c r="T55" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>375</v>
+      </c>
+      <c r="B56" t="s">
+        <v>290</v>
+      </c>
+      <c r="C56" t="s">
+        <v>410</v>
+      </c>
+      <c r="D56">
+        <v>282.02</v>
+      </c>
+      <c r="E56">
+        <v>0.24299999999999999</v>
+      </c>
+      <c r="F56">
+        <v>7.5</v>
+      </c>
+      <c r="L56">
+        <v>500</v>
+      </c>
+      <c r="N56">
+        <v>0.3</v>
+      </c>
+      <c r="O56">
+        <v>180</v>
+      </c>
+      <c r="P56">
+        <v>328.15</v>
+      </c>
+      <c r="R56">
+        <v>1268</v>
+      </c>
+      <c r="S56" t="s">
+        <v>185</v>
+      </c>
+      <c r="T56" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>375</v>
+      </c>
+      <c r="B57" t="s">
+        <v>290</v>
+      </c>
+      <c r="C57" t="s">
+        <v>410</v>
+      </c>
+      <c r="D57">
+        <v>67.81</v>
+      </c>
+      <c r="E57">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="F57">
+        <v>7.8</v>
+      </c>
+      <c r="L57">
+        <v>200</v>
+      </c>
+      <c r="N57">
+        <v>0.2</v>
+      </c>
+      <c r="O57">
+        <v>180</v>
+      </c>
+      <c r="P57">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="R57">
+        <v>108</v>
+      </c>
+      <c r="S57" t="s">
+        <v>185</v>
+      </c>
+      <c r="T57" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>375</v>
+      </c>
+      <c r="B58" t="s">
+        <v>290</v>
+      </c>
+      <c r="C58" t="s">
+        <v>410</v>
+      </c>
+      <c r="D58">
+        <v>67.81</v>
+      </c>
+      <c r="E58">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="F58">
+        <v>7.8</v>
+      </c>
+      <c r="M58">
+        <v>0.2</v>
+      </c>
+      <c r="N58">
+        <v>180</v>
+      </c>
+      <c r="O58">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="Q58">
+        <v>129</v>
+      </c>
+      <c r="R58" t="s">
+        <v>412</v>
+      </c>
+      <c r="S58" t="s">
+        <v>416</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>375</v>
+      </c>
+      <c r="B59" t="s">
+        <v>290</v>
+      </c>
+      <c r="C59" t="s">
+        <v>410</v>
+      </c>
+      <c r="D59">
+        <v>67.81</v>
+      </c>
+      <c r="E59">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="F59">
+        <v>7.8</v>
+      </c>
+      <c r="L59">
+        <v>200</v>
+      </c>
+      <c r="N59">
+        <v>0.2</v>
+      </c>
+      <c r="O59">
+        <v>180</v>
+      </c>
+      <c r="P59">
+        <v>298.14999999999998</v>
+      </c>
+      <c r="R59">
+        <v>108</v>
+      </c>
+      <c r="S59" t="s">
+        <v>185</v>
+      </c>
+      <c r="T59" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>375</v>
+      </c>
+      <c r="B60" t="s">
+        <v>290</v>
+      </c>
+      <c r="C60" t="s">
+        <v>410</v>
+      </c>
+      <c r="D60">
+        <v>67.81</v>
+      </c>
+      <c r="E60">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="F60">
+        <v>7.8</v>
+      </c>
+      <c r="L60">
+        <v>200</v>
+      </c>
+      <c r="N60">
+        <v>0.2</v>
+      </c>
+      <c r="O60">
+        <v>180</v>
+      </c>
+      <c r="P60">
+        <v>308.14999999999998</v>
+      </c>
+      <c r="R60">
+        <v>184</v>
+      </c>
+      <c r="S60" t="s">
+        <v>185</v>
+      </c>
+      <c r="T60" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>375</v>
+      </c>
+      <c r="B61" t="s">
+        <v>290</v>
+      </c>
+      <c r="C61" t="s">
+        <v>410</v>
+      </c>
+      <c r="D61">
+        <v>67.81</v>
+      </c>
+      <c r="E61">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="F61">
+        <v>7.8</v>
+      </c>
+      <c r="L61">
+        <v>200</v>
+      </c>
+      <c r="N61">
+        <v>0.2</v>
+      </c>
+      <c r="O61">
+        <v>180</v>
+      </c>
+      <c r="P61">
+        <v>318.14999999999998</v>
+      </c>
+      <c r="R61">
+        <v>361</v>
+      </c>
+      <c r="S61" t="s">
+        <v>185</v>
+      </c>
+      <c r="T61" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>375</v>
+      </c>
+      <c r="B62" t="s">
+        <v>290</v>
+      </c>
+      <c r="C62" t="s">
+        <v>410</v>
+      </c>
+      <c r="D62">
+        <v>67.81</v>
+      </c>
+      <c r="E62">
+        <v>0.13600000000000001</v>
+      </c>
+      <c r="F62">
+        <v>7.8</v>
+      </c>
+      <c r="L62">
+        <v>200</v>
+      </c>
+      <c r="N62">
+        <v>0.2</v>
+      </c>
+      <c r="O62">
+        <v>180</v>
+      </c>
+      <c r="P62">
+        <v>328.15</v>
+      </c>
+      <c r="R62">
+        <v>897</v>
+      </c>
+      <c r="S62" t="s">
+        <v>185</v>
+      </c>
+      <c r="T62" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>381</v>
+      </c>
+      <c r="B63" t="s">
+        <v>290</v>
+      </c>
+      <c r="C63" t="s">
+        <v>453</v>
+      </c>
+      <c r="D63">
+        <v>117</v>
+      </c>
+      <c r="E63">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="F63">
+        <v>7.79</v>
+      </c>
+      <c r="M63">
+        <v>0.4</v>
+      </c>
+      <c r="N63">
+        <v>1440</v>
+      </c>
+      <c r="O63">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="Q63">
+        <v>29</v>
+      </c>
+      <c r="R63" t="s">
+        <v>185</v>
+      </c>
+      <c r="S63" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>381</v>
+      </c>
+      <c r="B64" t="s">
+        <v>290</v>
+      </c>
+      <c r="C64" t="s">
+        <v>455</v>
+      </c>
+      <c r="D64">
+        <v>146</v>
+      </c>
+      <c r="E64">
+        <v>0.187</v>
+      </c>
+      <c r="F64">
+        <v>7.68</v>
+      </c>
+      <c r="M64">
+        <v>0.4</v>
+      </c>
+      <c r="N64">
+        <v>1440</v>
+      </c>
+      <c r="O64">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="Q64">
+        <v>23</v>
+      </c>
+      <c r="R64" t="s">
+        <v>185</v>
+      </c>
+      <c r="S64" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="65" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>381</v>
+      </c>
+      <c r="B65" t="s">
+        <v>290</v>
+      </c>
+      <c r="C65" t="s">
+        <v>453</v>
+      </c>
+      <c r="D65">
+        <v>154</v>
+      </c>
+      <c r="E65">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="F65">
+        <v>7.33</v>
+      </c>
+      <c r="M65">
+        <v>0.4</v>
+      </c>
+      <c r="N65">
+        <v>1440</v>
+      </c>
+      <c r="O65">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="Q65">
+        <v>32</v>
+      </c>
+      <c r="R65" t="s">
+        <v>185</v>
+      </c>
+      <c r="S65" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="66" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>381</v>
+      </c>
+      <c r="B66" t="s">
+        <v>290</v>
+      </c>
+      <c r="C66" t="s">
+        <v>455</v>
+      </c>
+      <c r="D66">
+        <v>109</v>
+      </c>
+      <c r="E66">
+        <v>0.15</v>
+      </c>
+      <c r="F66">
+        <v>6.98</v>
+      </c>
+      <c r="M66">
+        <v>0.4</v>
+      </c>
+      <c r="N66">
+        <v>1440</v>
+      </c>
+      <c r="O66">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="Q66">
+        <v>19</v>
+      </c>
+      <c r="R66" t="s">
+        <v>185</v>
+      </c>
+      <c r="S66" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="67" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A67" t="s">
+        <v>381</v>
+      </c>
+      <c r="B67" t="s">
+        <v>290</v>
+      </c>
+      <c r="C67" t="s">
+        <v>453</v>
+      </c>
+      <c r="D67">
+        <v>117</v>
+      </c>
+      <c r="E67">
+        <v>0.23899999999999999</v>
+      </c>
+      <c r="F67">
+        <v>7.79</v>
+      </c>
+      <c r="K67">
+        <v>20</v>
+      </c>
+      <c r="M67">
+        <v>0.4</v>
+      </c>
+      <c r="N67">
+        <v>1440</v>
+      </c>
+      <c r="O67">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="P67">
+        <v>10</v>
+      </c>
+      <c r="Q67">
+        <v>25</v>
+      </c>
+      <c r="R67" t="s">
+        <v>185</v>
+      </c>
+      <c r="S67" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="68" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>381</v>
+      </c>
+      <c r="B68" t="s">
+        <v>290</v>
+      </c>
+      <c r="C68" t="s">
+        <v>455</v>
+      </c>
+      <c r="D68">
+        <v>146</v>
+      </c>
+      <c r="E68">
+        <v>0.187</v>
+      </c>
+      <c r="F68">
+        <v>7.68</v>
+      </c>
+      <c r="K68">
+        <v>20</v>
+      </c>
+      <c r="M68">
+        <v>0.4</v>
+      </c>
+      <c r="N68">
+        <v>1440</v>
+      </c>
+      <c r="O68">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="P68">
+        <v>10.8</v>
+      </c>
+      <c r="Q68">
+        <v>23</v>
+      </c>
+      <c r="R68" t="s">
+        <v>185</v>
+      </c>
+      <c r="S68" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="69" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>381</v>
+      </c>
+      <c r="B69" t="s">
+        <v>290</v>
+      </c>
+      <c r="C69" t="s">
+        <v>453</v>
+      </c>
+      <c r="D69">
+        <v>154</v>
+      </c>
+      <c r="E69">
+        <v>0.24099999999999999</v>
+      </c>
+      <c r="F69">
+        <v>7.33</v>
+      </c>
+      <c r="K69">
+        <v>20</v>
+      </c>
+      <c r="M69">
+        <v>0.4</v>
+      </c>
+      <c r="N69">
+        <v>1440</v>
+      </c>
+      <c r="O69">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="P69">
+        <v>7.2</v>
+      </c>
+      <c r="Q69">
+        <v>32</v>
+      </c>
+      <c r="R69" t="s">
+        <v>185</v>
+      </c>
+      <c r="S69" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="70" spans="1:19" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>381</v>
+      </c>
+      <c r="B70" t="s">
+        <v>290</v>
+      </c>
+      <c r="C70" t="s">
+        <v>455</v>
+      </c>
+      <c r="D70">
+        <v>109</v>
+      </c>
+      <c r="E70">
+        <v>0.15</v>
+      </c>
+      <c r="F70">
+        <v>6.98</v>
+      </c>
+      <c r="K70">
+        <v>20</v>
+      </c>
+      <c r="M70">
+        <v>0.4</v>
+      </c>
+      <c r="N70">
+        <v>1440</v>
+      </c>
+      <c r="O70">
+        <v>295.14999999999998</v>
+      </c>
+      <c r="P70">
+        <v>13.2</v>
+      </c>
+      <c r="Q70">
+        <v>17</v>
+      </c>
+      <c r="R70" t="s">
+        <v>185</v>
+      </c>
+      <c r="S70" t="s">
+        <v>462</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E26"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>